<commit_message>
Itinerary: outbound flights via Beijing, updated hotel prices
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GRL2UxCPJBrQ7CY9ADTFYy
</commit_message>
<xml_diff>
--- a/visseo.info-site/itinerary/China_Trip_2026.xlsx
+++ b/visseo.info-site/itinerary/China_Trip_2026.xlsx
@@ -26,12 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="210">
   <si>
     <t xml:space="preserve">China &amp; Hong Kong 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">30 Oct – 23 Nov 2026  ·  25 days  ·  Shenzhen → Hong Kong → Guangzhou → Zhangjiajie → Chongqing → Chengdu → Chongqing  ·  all by train</t>
+    <t xml:space="preserve">30 Oct – 23 Nov 2026  ·  25 days  ·  via Beijing  ·  Shenzhen → Hong Kong → Guangzhou → Zhangjiajie → Chongqing → Chengdu → Chongqing  ·  all by train</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -67,8 +67,7 @@
     <t xml:space="preserve">✈️ Flight</t>
   </si>
   <si>
-    <t xml:space="preserve">Flight: Brussels (BRU) -&gt; Shenzhen (SZX) 
-Dep: 10:40 AM 
+    <t xml:space="preserve">Flight HU492 Brussels (BRU) 12:20 → Beijing (PEK, T2) 04:40 next morning
 Overnight flight</t>
   </si>
   <si>
@@ -78,22 +77,13 @@
     <t xml:space="preserve">In-flight meals</t>
   </si>
   <si>
-    <t xml:space="preserve">Rest and prepare flight logistics.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In-flight relaxation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long-haul travel preparation.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sat</t>
   </si>
   <si>
     <t xml:space="preserve">Shenzhen</t>
   </si>
   <si>
-    <t xml:space="preserve">Arrival 05:00 AM at SZX. Drop bags at the hotel, rest/breakfast, then Futian (≈35 min by metro/taxi): Huaqiangbei to buy the camera (shops open ≈10:00), Lianhuashan Park nearby, evening in Futian.</t>
+    <t xml:space="preserve">Flight HU7701 Beijing (PEK, T2) 08:30 → Shenzhen (SZX, T3) 11:55 – immigration &amp; customs happen in Beijing. Hotel ≈13:00 (≈25 min), then Futian (≈35 min): Huaqiangbei to buy the camera, Lianhuashan Park nearby, evening in Futian.</t>
   </si>
   <si>
     <t xml:space="preserve">Pagoda SSAW</t>
@@ -1501,13 +1491,25 @@
     <t xml:space="preserve">Booked?</t>
   </si>
   <si>
+    <t xml:space="preserve">✈️ Flight HU492</t>
+  </si>
+  <si>
     <t xml:space="preserve">Brussels (BRU)</t>
   </si>
   <si>
-    <t xml:space="preserve">Shenzhen (SZX)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dep 10:40 → arr 31 Oct ≈05:00</t>
+    <t xml:space="preserve">Beijing (PEK) T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dep 12:20 → arr 31 Oct 04:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✈️ Flight HU7701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shenzhen (SZX) T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dep 08:30 → arr 11:55</t>
   </si>
   <si>
     <t xml:space="preserve">🚄 Train</t>
@@ -2553,43 +2555,37 @@
       <c r="F6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="n">
         <v>46326</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="F7" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="G7" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="H7" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="I7" s="13" t="s">
         <v>23</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2597,28 +2593,28 @@
         <v>46327</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="H8" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="8" t="s">
+      <c r="I8" s="8" t="s">
         <v>29</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2626,28 +2622,28 @@
         <v>46328</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="12" t="s">
+      <c r="H9" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>35</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2655,28 +2651,28 @@
         <v>46329</v>
       </c>
       <c r="B10" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="F10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="H10" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="I10" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2684,28 +2680,28 @@
         <v>46330</v>
       </c>
       <c r="B11" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="17" t="s">
+      <c r="H11" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" s="18" t="s">
+      <c r="I11" s="18" t="s">
         <v>49</v>
-      </c>
-      <c r="G11" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="H11" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="I11" s="18" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2713,28 +2709,28 @@
         <v>46331</v>
       </c>
       <c r="B12" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="H12" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="8" t="s">
+      <c r="I12" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2745,25 +2741,25 @@
         <v>11</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D13" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H13" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="13" t="s">
+      <c r="I13" s="13" t="s">
         <v>60</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="H13" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="I13" s="13" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2771,28 +2767,28 @@
         <v>46333</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H14" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E14" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="8" t="s">
+      <c r="I14" s="8" t="s">
         <v>65</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2800,28 +2796,28 @@
         <v>46334</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C15" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="G15" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="H15" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="I15" s="13" t="s">
         <v>72</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2829,28 +2825,28 @@
         <v>46335</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C16" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="H16" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" s="8" t="s">
+      <c r="I16" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2858,28 +2854,28 @@
         <v>46336</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D17" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="H17" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="E17" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F17" s="13" t="s">
+      <c r="I17" s="13" t="s">
         <v>83</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="I17" s="13" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2887,28 +2883,28 @@
         <v>46337</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C18" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="G18" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="H18" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="I18" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="I18" s="8" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2916,28 +2912,28 @@
         <v>46338</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C19" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="H19" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="E19" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="F19" s="13" t="s">
+      <c r="I19" s="13" t="s">
         <v>96</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="I19" s="13" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2948,25 +2944,25 @@
         <v>11</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D20" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="H20" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F20" s="8" t="s">
+      <c r="I20" s="8" t="s">
         <v>101</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2974,28 +2970,28 @@
         <v>46340</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C21" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F21" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="G21" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="H21" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="I21" s="13" t="s">
         <v>108</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="H21" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="I21" s="13" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3003,28 +2999,28 @@
         <v>46341</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C22" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="G22" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="H22" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="E22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="F22" s="28" t="s">
+      <c r="I22" s="8" t="s">
         <v>114</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3032,28 +3028,28 @@
         <v>46342</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D23" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="H23" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="E23" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="F23" s="13" t="s">
+      <c r="I23" s="13" t="s">
         <v>119</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="H23" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="I23" s="13" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3061,28 +3057,28 @@
         <v>46343</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D24" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="H24" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="E24" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="F24" s="8" t="s">
+      <c r="I24" s="8" t="s">
         <v>124</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3090,28 +3086,28 @@
         <v>46344</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C25" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="F25" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="G25" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="H25" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="F25" s="13" t="s">
+      <c r="I25" s="13" t="s">
         <v>131</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H25" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="I25" s="13" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3119,28 +3115,28 @@
         <v>46345</v>
       </c>
       <c r="B26" s="30" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C26" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="G26" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="H26" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E26" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="F26" s="8" t="s">
+      <c r="I26" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3151,25 +3147,25 @@
         <v>11</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D27" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="H27" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="E27" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="F27" s="13" t="s">
+      <c r="I27" s="13" t="s">
         <v>142</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="H27" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3177,28 +3173,28 @@
         <v>46347</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C28" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="F28" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="G28" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="H28" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="I28" s="8" t="s">
         <v>149</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3206,28 +3202,28 @@
         <v>46348</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D29" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G29" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="H29" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="E29" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="F29" s="13" t="s">
+      <c r="I29" s="13" t="s">
         <v>154</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="H29" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="I29" s="13" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3235,13 +3231,13 @@
         <v>46349</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>14</v>
@@ -3250,13 +3246,13 @@
         <v>15</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -3291,12 +3287,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3307,30 +3303,30 @@
         <v>6</v>
       </c>
       <c r="C4" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="F4" s="33" t="s">
         <v>164</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="G4" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="H4" s="32" t="s">
         <v>166</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>167</v>
-      </c>
-      <c r="G4" s="33" t="s">
-        <v>168</v>
-      </c>
-      <c r="H4" s="32" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C5" s="36" t="n">
         <v>46326</v>
@@ -3343,22 +3339,22 @@
         <v>3</v>
       </c>
       <c r="F5" s="38" t="n">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="G5" s="38" t="n">
         <f aca="false">IFERROR(F5/E5,"")</f>
-        <v>68.6666666666667</v>
+        <v>71.6666666666667</v>
       </c>
       <c r="H5" s="35" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="39" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C6" s="36" t="n">
         <v>46329</v>
@@ -3371,22 +3367,22 @@
         <v>5</v>
       </c>
       <c r="F6" s="38" t="n">
-        <v>900</v>
+        <v>921</v>
       </c>
       <c r="G6" s="38" t="n">
         <f aca="false">IFERROR(F6/E6,"")</f>
-        <v>180</v>
+        <v>184.2</v>
       </c>
       <c r="H6" s="35" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="40" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>46334</v>
@@ -3399,22 +3395,22 @@
         <v>3</v>
       </c>
       <c r="F7" s="38" t="n">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="G7" s="38" t="n">
         <f aca="false">IFERROR(F7/E7,"")</f>
-        <v>83.3333333333333</v>
+        <v>86.3333333333333</v>
       </c>
       <c r="H7" s="35" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C8" s="36" t="n">
         <v>46337</v>
@@ -3434,15 +3430,15 @@
         <v>118.333333333333</v>
       </c>
       <c r="H8" s="35" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="42" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C9" s="36" t="n">
         <v>46340</v>
@@ -3462,15 +3458,15 @@
         <v>76.25</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>46344</v>
@@ -3490,15 +3486,15 @@
         <v>58</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="42" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C11" s="36" t="n">
         <v>46347</v>
@@ -3518,12 +3514,12 @@
         <v>96.5</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="44" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B12" s="44"/>
       <c r="C12" s="45"/>
@@ -3534,14 +3530,14 @@
       </c>
       <c r="F12" s="47" t="n">
         <f aca="false">SUM(F5:F11)</f>
-        <v>2383</v>
+        <v>2422</v>
       </c>
       <c r="G12" s="47" t="n">
         <f aca="false">F12/E12</f>
-        <v>103.608695652174</v>
+        <v>105.304347826087</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -3560,7 +3556,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -3572,12 +3568,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3585,19 +3581,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="48" t="s">
+        <v>178</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>179</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>180</v>
+      </c>
+      <c r="E4" s="48" t="s">
         <v>181</v>
       </c>
-      <c r="C4" s="48" t="s">
+      <c r="F4" s="48" t="s">
         <v>182</v>
-      </c>
-      <c r="D4" s="48" t="s">
-        <v>183</v>
-      </c>
-      <c r="E4" s="48" t="s">
-        <v>184</v>
-      </c>
-      <c r="F4" s="48" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3605,85 +3601,85 @@
         <v>46325</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>12</v>
+        <v>183</v>
       </c>
       <c r="C5" s="50" t="s">
+        <v>184</v>
+      </c>
+      <c r="D5" s="50" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" s="50" t="s">
         <v>186</v>
-      </c>
-      <c r="D5" s="50" t="s">
-        <v>187</v>
-      </c>
-      <c r="E5" s="50" t="s">
-        <v>188</v>
       </c>
       <c r="F5" s="51"/>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="52" t="n">
-        <v>46329</v>
+        <v>46326</v>
       </c>
       <c r="B6" s="53" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="53" t="s">
         <v>189</v>
-      </c>
-      <c r="C6" s="53" t="s">
-        <v>190</v>
-      </c>
-      <c r="D6" s="53" t="s">
-        <v>191</v>
-      </c>
-      <c r="E6" s="53" t="s">
-        <v>192</v>
       </c>
       <c r="F6" s="54"/>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="49" t="n">
-        <v>46334</v>
+        <v>46329</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>191</v>
       </c>
       <c r="D7" s="50" t="s">
+        <v>192</v>
+      </c>
+      <c r="E7" s="50" t="s">
         <v>193</v>
-      </c>
-      <c r="E7" s="50" t="s">
-        <v>194</v>
       </c>
       <c r="F7" s="51"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="52" t="n">
-        <v>46337</v>
+        <v>46334</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C8" s="53" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D8" s="53" t="s">
+        <v>194</v>
+      </c>
+      <c r="E8" s="53" t="s">
         <v>195</v>
-      </c>
-      <c r="E8" s="53" t="s">
-        <v>196</v>
       </c>
       <c r="F8" s="54"/>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="49" t="n">
-        <v>46340</v>
+        <v>46337</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D9" s="50" t="s">
-        <v>112</v>
+        <v>196</v>
       </c>
       <c r="E9" s="50" t="s">
         <v>197</v>
@@ -3692,93 +3688,111 @@
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="52" t="n">
-        <v>46342</v>
+        <v>46340</v>
       </c>
       <c r="B10" s="53" t="s">
+        <v>190</v>
+      </c>
+      <c r="C10" s="53" t="s">
+        <v>196</v>
+      </c>
+      <c r="D10" s="53" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="53" t="s">
         <v>198</v>
-      </c>
-      <c r="C10" s="53" t="s">
-        <v>112</v>
-      </c>
-      <c r="D10" s="53" t="s">
-        <v>199</v>
-      </c>
-      <c r="E10" s="53" t="s">
-        <v>200</v>
       </c>
       <c r="F10" s="54"/>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="49" t="n">
-        <v>46344</v>
+        <v>46342</v>
       </c>
       <c r="B11" s="50" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D11" s="50" t="s">
+        <v>200</v>
+      </c>
+      <c r="E11" s="50" t="s">
         <v>201</v>
-      </c>
-      <c r="E11" s="50" t="s">
-        <v>202</v>
       </c>
       <c r="F11" s="51"/>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="52" t="n">
-        <v>46346</v>
+        <v>46344</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C12" s="53" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" s="53" t="s">
+        <v>202</v>
+      </c>
+      <c r="E12" s="53" t="s">
         <v>203</v>
-      </c>
-      <c r="D12" s="53" t="s">
-        <v>204</v>
-      </c>
-      <c r="E12" s="53" t="s">
-        <v>205</v>
       </c>
       <c r="F12" s="54"/>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="49" t="n">
-        <v>46347</v>
+        <v>46346</v>
       </c>
       <c r="B13" s="50" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D13" s="50" t="s">
-        <v>112</v>
+        <v>205</v>
       </c>
       <c r="E13" s="50" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="F13" s="51"/>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="52" t="n">
+        <v>46347</v>
+      </c>
+      <c r="B14" s="53" t="s">
+        <v>190</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>202</v>
+      </c>
+      <c r="D14" s="53" t="s">
+        <v>109</v>
+      </c>
+      <c r="E14" s="53" t="s">
+        <v>203</v>
+      </c>
+      <c r="F14" s="54"/>
+    </row>
+    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="49" t="n">
         <v>46349</v>
       </c>
-      <c r="B14" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="C14" s="53" t="s">
+      <c r="B15" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="D14" s="53" t="s">
-        <v>186</v>
-      </c>
-      <c r="E14" s="53" t="s">
+      <c r="C15" s="50" t="s">
         <v>208</v>
       </c>
-      <c r="F14" s="54"/>
+      <c r="D15" s="50" t="s">
+        <v>184</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>209</v>
+      </c>
+      <c r="F15" s="51"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>